<commit_message>
Registra a fatura de agosto: 705 kWh, a maior do historico
Leitura de 29/07 a 27/08, 29 dias, R$ 741,61. Sao 24,31 kWh/dia contra
16,36 em julho e 11,57 na casa estavel de antes de maio.

A projecao desta planilha era 603 kWh. Errou 17% para menos. Os 102 kWh
a mais tem duas explicacoes possiveis e a fatura sozinha nao separa:
ou o carro puxou 259 kWh da tomada (86% da bateria por dia, plausivel),
ou a casa deu mais um degrau e foi a 18,9 kWh/dia.

A fatura tambem confirma que o fornecimento segue MONOFASICO na leitura
de 27/08 - a adequacao para bifasico que o Anexo 1 ja declara nao foi
feita. Tarifa subiu cerca de 2% sobre julho e a COSIP subiu 25% por ser
escalonada no consumo. Entrou um bonus Itaipu de R$ 18,95.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G5xS2RAgiQC8EwtpN9vnAe
</commit_message>
<xml_diff>
--- a/solar/Comparativo_Orcamentos_Solar_Henrique.xlsx
+++ b/solar/Comparativo_Orcamentos_Solar_Henrique.xlsx
@@ -12599,7 +12599,7 @@
           <t>Jul/26</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n">
+      <c r="C18" s="11" t="n">
         <v>540</v>
       </c>
       <c r="D18" s="11" t="n">
@@ -12611,10 +12611,20 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Linha 6 = Jul/25 (mes mais antigo). Linha 18 = Jul/26 (mes atual). Verde = menor consumo. Vermelho = maior consumo.</t>
-        </is>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>Ago/26</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="n">
+        <v>705</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="E19" s="19">
+        <f>IFERROR(C19/D19,0)</f>
+        <v/>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -12623,6 +12633,11 @@
       </c>
     </row>
     <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Linha 6 = Jul/25 (mes mais antigo). Linha 19 = Ago/26 (mes atual). Verde = menor consumo. Vermelho = maior consumo.</t>
+        </is>
+      </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Distribuidora</t>
@@ -12661,7 +12676,7 @@
         </is>
       </c>
       <c r="C22" s="26">
-        <f>SUM(C7:C18)</f>
+        <f>SUM(C8:C19)</f>
         <v/>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -12713,7 +12728,7 @@
         </is>
       </c>
       <c r="C24" s="12">
-        <f>SUM(D7:D18)</f>
+        <f>SUM(D8:D19)</f>
         <v/>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -12761,11 +12776,11 @@
     <row r="26">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>MAIOR CONSUMO (Jul/26)</t>
+          <t>MAIOR CONSUMO (Ago/26)</t>
         </is>
       </c>
       <c r="C26" s="12">
-        <f>MAX(C7:C18)</f>
+        <f>MAX(C8:C19)</f>
         <v/>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -12791,7 +12806,7 @@
         </is>
       </c>
       <c r="C27" s="12">
-        <f>MIN(C7:C18)</f>
+        <f>MIN(C8:C19)</f>
         <v/>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -12835,11 +12850,11 @@
     <row r="29">
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Consumo do mes atual (Jul/26)</t>
+          <t>Consumo do mes atual (Ago/26)</t>
         </is>
       </c>
       <c r="C29" s="12">
-        <f>C18</f>
+        <f>C19</f>
         <v/>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -12887,7 +12902,7 @@
         </is>
       </c>
       <c r="C31" s="29">
-        <f>AVERAGE(C7:C12)</f>
+        <f>AVERAGE(C8:C13)</f>
         <v/>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -12913,7 +12928,7 @@
         </is>
       </c>
       <c r="C32" s="29">
-        <f>AVERAGE(C13:C18)</f>
+        <f>AVERAGE(C14:C19)</f>
         <v/>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -12961,11 +12976,11 @@
     <row r="34">
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>MESMO MES, ANO ANTERIOR: Jul/25 x Jul/26</t>
+          <t>MESMO MES, ANO ANTERIOR: Ago/25 x Ago/26</t>
         </is>
       </c>
       <c r="C34" s="31">
-        <f>IFERROR(C18/C6-1,0)</f>
+        <f>IFERROR(C19/C7-1,0)</f>
         <v/>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -13397,7 +13412,7 @@
         </is>
       </c>
       <c r="C78" s="29">
-        <f>AVERAGE(E16:E18)</f>
+        <f>AVERAGE(E16:E19)</f>
         <v/>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -13469,11 +13484,11 @@
     <row r="82">
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>CONTROLE DE SAZONALIDADE - Jul/25</t>
+          <t>CONTROLE DE SAZONALIDADE - Ago/25</t>
         </is>
       </c>
       <c r="C82" s="29">
-        <f>E6</f>
+        <f>E7</f>
         <v/>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -13490,11 +13505,11 @@
     <row r="83">
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>CONTROLE DE SAZONALIDADE - Jul/26</t>
+          <t>CONTROLE DE SAZONALIDADE - Ago/25 x Ago/26</t>
         </is>
       </c>
       <c r="C83" s="29">
-        <f>E18</f>
+        <f>E19</f>
         <v/>
       </c>
       <c r="D83" s="2" t="inlineStr">

</xml_diff>